<commit_message>
CI Reports [2026-07-01 08:47]: CreateTicket — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S26"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -540,9 +540,1473 @@
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
       </c>
     </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TC-CT-001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Submit valid ticket with all required fields</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>API</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H3" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I3" t="str">
+        <v>BUG-CREATETICKET-002</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Submit valid ticket with all required fields</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L3" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M3" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-001
+3. Observe failure</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R3" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S3" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C4" t="str">
+        <v>TC-CT-002</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Submit valid ticket with optional Page/Screen Name</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>API</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H4" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I4" t="str">
+        <v>BUG-CREATETICKET-003</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Submit valid ticket with optional Page/Screen Name</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M4" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-002
+3. Observe failure</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R4" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TC-CT-003</v>
+      </c>
+      <c r="D5" t="str">
+        <v>All 6 ticket type chips are individually selectable</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H5" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I5" t="str">
+        <v>BUG-CREATETICKET-004</v>
+      </c>
+      <c r="J5" t="str">
+        <v>All 6 ticket type chips are individually selectable</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L5" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M5" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-003
+3. Observe failure</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R5" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C6" t="str">
+        <v>TC-CT-004</v>
+      </c>
+      <c r="D6" t="str">
+        <v>All platform chips are individually selectable</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I6" t="str">
+        <v>BUG-CREATETICKET-005</v>
+      </c>
+      <c r="J6" t="str">
+        <v>All platform chips are individually selectable</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L6" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M6" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-004
+3. Observe failure</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R6" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TC-CT-005</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Reset button shows confirmation and clears all form fields</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F7" t="str">
+        <v>API</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H7" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I7" t="str">
+        <v>BUG-CREATETICKET-006</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Reset button shows confirmation and clears all form fields</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L7" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M7" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-005
+3. Observe failure</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R7" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C8" t="str">
+        <v>TC-CT-006</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Character counter updates dynamically as user types</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>API</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H8" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I8" t="str">
+        <v>BUG-CREATETICKET-007</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Character counter updates dynamically as user types</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L8" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M8" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-006
+3. Observe failure</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R8" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TC-CT-007</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Page loads with correct title, heading and all UI elements</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H9" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I9" t="str">
+        <v>BUG-CREATETICKET-008</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Page loads with correct title, heading and all UI elements</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L9" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M9" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-007
+3. Observe failure</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R9" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S9" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C10" t="str">
+        <v>TC-CT-008</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Submit without project shows validation error</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>API</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H10" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I10" t="str">
+        <v>BUG-CREATETICKET-009</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Submit without project shows validation error</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L10" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M10" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-008
+3. Observe failure</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R10" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C11" t="str">
+        <v>TC-CT-009</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Submit without ticket type shows validation error</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>API</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H11" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I11" t="str">
+        <v>BUG-CREATETICKET-010</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Submit without ticket type shows validation error</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L11" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M11" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-009
+3. Observe failure</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R11" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S11" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C12" t="str">
+        <v>TC-CT-010</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Submit without platform shows validation error</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>API</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H12" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I12" t="str">
+        <v>BUG-CREATETICKET-011</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Submit without platform shows validation error</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L12" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M12" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-010
+3. Observe failure</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R12" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S12" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C13" t="str">
+        <v>TC-CT-011</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Submit without description shows validation error</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F13" t="str">
+        <v>API</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H13" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I13" t="str">
+        <v>BUG-CREATETICKET-012</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Submit without description shows validation error</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L13" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M13" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-011
+3. Observe failure</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R13" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S13" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C14" t="str">
+        <v>TC-CT-012</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Submit with description below 15 chars is rejected</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F14" t="str">
+        <v>API</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H14" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I14" t="str">
+        <v>BUG-CREATETICKET-013</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Submit with description below 15 chars is rejected</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L14" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M14" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-012
+3. Observe failure</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R14" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S14" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C15" t="str">
+        <v>TC-CT-013</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Submit all fields empty shows all validation errors</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G15" t="str">
+        <v>High</v>
+      </c>
+      <c r="H15" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I15" t="str">
+        <v>BUG-CREATETICKET-014</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Submit all fields empty shows all validation errors</v>
+      </c>
+      <c r="K15" t="str">
+        <v>High</v>
+      </c>
+      <c r="L15" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M15" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-013
+3. Observe failure</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R15" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S15" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C16" t="str">
+        <v>TC-CT-014</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Description exactly 15 chars (min boundary) is accepted</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F16" t="str">
+        <v>API</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H16" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I16" t="str">
+        <v>BUG-CREATETICKET-015</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Description exactly 15 chars (min boundary) is accepted</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L16" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M16" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-014
+3. Observe failure</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R16" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S16" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C17" t="str">
+        <v>TC-CT-015</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Description exactly 14 chars (below min) is rejected</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F17" t="str">
+        <v>API</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H17" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I17" t="str">
+        <v>BUG-CREATETICKET-016</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Description exactly 14 chars (below min) is rejected</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L17" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M17" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-015
+3. Observe failure</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R17" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S17" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C18" t="str">
+        <v>TC-CT-016</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Description exactly 2000 chars (max boundary) is accepted</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F18" t="str">
+        <v>API</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H18" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>BUG-CREATETICKET-017</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Description exactly 2000 chars (max boundary) is accepted</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L18" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M18" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-016
+3. Observe failure</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R18" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S18" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C19" t="str">
+        <v>TC-CT-017</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Description 2001 chars should be blocked — BUG-CT-001</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F19" t="str">
+        <v>API</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H19" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I19" t="str">
+        <v>BUG-CREATETICKET-018</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Description 2001 chars should be blocked — BUG-CT-001</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L19" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M19" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-017
+3. Observe failure</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R19" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S19" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C20" t="str">
+        <v>TC-CT-018</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Page/Screen Name 300 chars handled gracefully</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F20" t="str">
+        <v>API</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H20" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I20" t="str">
+        <v>BUG-CREATETICKET-019</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Page/Screen Name 300 chars handled gracefully</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L20" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M20" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-018
+3. Observe failure</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R20" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S20" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C21" t="str">
+        <v>TC-CT-019</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Unauthenticated access redirects to login</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G21" t="str">
+        <v>High</v>
+      </c>
+      <c r="H21" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I21" t="str">
+        <v>BUG-CREATETICKET-020</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Unauthenticated access redirects to login</v>
+      </c>
+      <c r="K21" t="str">
+        <v>High</v>
+      </c>
+      <c r="L21" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M21" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-019
+3. Observe failure</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R21" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S21" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C22" t="str">
+        <v>TC-CT-020</v>
+      </c>
+      <c r="D22" t="str">
+        <v>SQL injection in description handled safely</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F22" t="str">
+        <v>API</v>
+      </c>
+      <c r="G22" t="str">
+        <v>High</v>
+      </c>
+      <c r="H22" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I22" t="str">
+        <v>BUG-CREATETICKET-021</v>
+      </c>
+      <c r="J22" t="str">
+        <v>SQL injection in description handled safely</v>
+      </c>
+      <c r="K22" t="str">
+        <v>High</v>
+      </c>
+      <c r="L22" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M22" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-020
+3. Observe failure</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R22" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S22" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C23" t="str">
+        <v>TC-CT-021</v>
+      </c>
+      <c r="D23" t="str">
+        <v>XSS payload in description does not execute</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F23" t="str">
+        <v>API</v>
+      </c>
+      <c r="G23" t="str">
+        <v>High</v>
+      </c>
+      <c r="H23" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I23" t="str">
+        <v>BUG-CREATETICKET-022</v>
+      </c>
+      <c r="J23" t="str">
+        <v>XSS payload in description does not execute</v>
+      </c>
+      <c r="K23" t="str">
+        <v>High</v>
+      </c>
+      <c r="L23" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M23" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-021
+3. Observe failure</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R23" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S23" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C24" t="str">
+        <v>TC-CT-022</v>
+      </c>
+      <c r="D24" t="str">
+        <v>HTML injection in description is sanitised</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F24" t="str">
+        <v>API</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H24" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I24" t="str">
+        <v>BUG-CREATETICKET-023</v>
+      </c>
+      <c r="J24" t="str">
+        <v>HTML injection in description is sanitised</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L24" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M24" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-022
+3. Observe failure</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R24" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C25" t="str">
+        <v>TC-CT-023</v>
+      </c>
+      <c r="D25" t="str">
+        <v>XSS payload in Page/Screen Name does not execute</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F25" t="str">
+        <v>API</v>
+      </c>
+      <c r="G25" t="str">
+        <v>High</v>
+      </c>
+      <c r="H25" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I25" t="str">
+        <v>BUG-CREATETICKET-024</v>
+      </c>
+      <c r="J25" t="str">
+        <v>XSS payload in Page/Screen Name does not execute</v>
+      </c>
+      <c r="K25" t="str">
+        <v>High</v>
+      </c>
+      <c r="L25" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M25" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-023
+3. Observe failure</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R25" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S25" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C26" t="str">
+        <v>TC-CT-024</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Cancel Reset dialog retains all form fields</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F26" t="str">
+        <v>API</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H26" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I26" t="str">
+        <v>BUG-CREATETICKET-025</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Cancel Reset dialog retains all form fields</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L26" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M26" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to CreateTicket feature
+2. Execute: TC-CT-024
+3. Observe failure</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R26" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S26" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 15:37]: Login — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:S27"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2004,9 +2004,68 @@
         <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Login</v>
+      </c>
+      <c r="C27" t="str">
+        <v>TC-LOGIN-001-summary</v>
+      </c>
+      <c r="D27" t="str">
+        <v>All 20 TCs passed — Login module</v>
+      </c>
+      <c r="E27" t="str">
+        <v>All types</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Unit / API / Auto</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Critical–Low</v>
+      </c>
+      <c r="H27" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I27" t="str">
+        <v>—</v>
+      </c>
+      <c r="J27" t="str">
+        <v>No bugs — 20/20 TCs passed</v>
+      </c>
+      <c r="K27" t="str">
+        <v>—</v>
+      </c>
+      <c r="L27" t="str">
+        <v>—</v>
+      </c>
+      <c r="M27" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P27" t="str">
+        <v>20 TCs via Playwright (tests/login.spec.js)</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>All 20 TCs pass</v>
+      </c>
+      <c r="R27" t="str">
+        <v>20/20 PASS ✓  Pass Rate: 100%</v>
+      </c>
+      <c r="S27" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 17:53]: AddNewUser — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S41"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2063,9 +2063,864 @@
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
       </c>
     </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C28" t="str">
+        <v>TC-AU-007</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Page loads with heading, stats, grid, Add New User button</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H28" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I28" t="str">
+        <v>BUG-ADDNEWUSER-026</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Page loads with heading, stats, grid, Add New User button</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L28" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M28" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to page
+2. Check h1, button, grid presence</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>h1='User Management'; addBtn visible; grid with user rows; stat cards shown</v>
+      </c>
+      <c r="R28" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S28" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C29" t="str">
+        <v>TC-AU-001</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Create Partner Admin — Automatic password</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F29" t="str">
+        <v>API</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H29" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I29" t="str">
+        <v>BUG-ADDNEWUSER-027</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Create Partner Admin — Automatic password</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L29" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M29" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O29" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open Add New User
+2. Fill all fields for Partner Admin
+3. Click Create User
+4. Check success feedback</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>'Success — Operation completed successfully.' shown; form resets; Partner Admin user created</v>
+      </c>
+      <c r="R29" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S29" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C30" t="str">
+        <v>TC-AU-002</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Create Partner User — Automatic password</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F30" t="str">
+        <v>API</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H30" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I30" t="str">
+        <v>BUG-ADDNEWUSER-028</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Create Partner User — Automatic password</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L30" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M30" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open modal
+2. Select Partner User role
+3. Check if Customer field is shown</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>Success feedback; Partner User created</v>
+      </c>
+      <c r="R30" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S30" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C31" t="str">
+        <v>TC-AU-003</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Create user with Manual password</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F31" t="str">
+        <v>API</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H31" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I31" t="str">
+        <v>BUG-ADDNEWUSER-029</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Create user with Manual password</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L31" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M31" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Manual radio
+2. Check #fPassword visibility
+3. Fill and submit</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>Password input visible when Manual selected; user created successfully</v>
+      </c>
+      <c r="R31" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S31" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C32" t="str">
+        <v>TC-AU-005</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Create user with Inactive status</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F32" t="str">
+        <v>API</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H32" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I32" t="str">
+        <v>BUG-ADDNEWUSER-030</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Create user with Inactive status</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L32" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M32" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select Inactive
+2. Submit
+3. Confirm status</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>User created with Inactive status; success feedback shown</v>
+      </c>
+      <c r="R32" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S32" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C33" t="str">
+        <v>TC-AU-008</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Cancel button closes modal without saving</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F33" t="str">
+        <v>API</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H33" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I33" t="str">
+        <v>BUG-ADDNEWUSER-031</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Cancel button closes modal without saving</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L33" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M33" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Fill some data
+2. Click Cancel
+3. Check modal state</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>Modal closes; filled data discarded; no user created</v>
+      </c>
+      <c r="R33" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S33" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B34" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C34" t="str">
+        <v>TC-AU-006</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Close (✕) button dismisses modal</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F34" t="str">
+        <v>API</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H34" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I34" t="str">
+        <v>BUG-ADDNEWUSER-032</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Close (✕) button dismisses modal</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L34" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M34" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O34" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Fill partial data
+2. Click ✕
+3. Check if modal closed</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>Modal closes; no user created; data discarded</v>
+      </c>
+      <c r="R34" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S34" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B35" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C35" t="str">
+        <v>TC-AU-019</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Single character First Name (min boundary) accepted</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F35" t="str">
+        <v>API</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H35" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I35" t="str">
+        <v>BUG-ADDNEWUSER-033</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Single character First Name (min boundary) accepted</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L35" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M35" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter "A" as First Name
+2. Submit
+3. Check if accepted</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>1-char First Name accepted; user created successfully</v>
+      </c>
+      <c r="R35" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S35" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B36" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C36" t="str">
+        <v>TC-AU-013</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Empty form submit shows all validation errors</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G36" t="str">
+        <v>High</v>
+      </c>
+      <c r="H36" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I36" t="str">
+        <v>BUG-ADDNEWUSER-034</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Empty form submit shows all validation errors</v>
+      </c>
+      <c r="K36" t="str">
+        <v>High</v>
+      </c>
+      <c r="L36" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M36" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open modal
+2. Click Create User immediately
+3. Check all error messages</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>All required field errors: First name, Username, Email, Role, Customer, Projects</v>
+      </c>
+      <c r="R36" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S36" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B37" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C37" t="str">
+        <v>TC-AU-010</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Empty First Name shows validation error</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G37" t="str">
+        <v>High</v>
+      </c>
+      <c r="H37" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I37" t="str">
+        <v>BUG-ADDNEWUSER-035</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Empty First Name shows validation error</v>
+      </c>
+      <c r="K37" t="str">
+        <v>High</v>
+      </c>
+      <c r="L37" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M37" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P37" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Leave First Name empty
+2. Submit
+3. Check wrapFirstName error</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>"First name is required" validation on #wrapFirstName; modal stays open</v>
+      </c>
+      <c r="R37" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S37" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B38" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C38" t="str">
+        <v>TC-AU-017</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Invalid email format shows validation error</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F38" t="str">
+        <v>API</v>
+      </c>
+      <c r="G38" t="str">
+        <v>High</v>
+      </c>
+      <c r="H38" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I38" t="str">
+        <v>BUG-ADDNEWUSER-036</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Invalid email format shows validation error</v>
+      </c>
+      <c r="K38" t="str">
+        <v>High</v>
+      </c>
+      <c r="L38" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M38" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P38" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter invalid email
+2. Submit
+3. Check email error message</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>"A valid email address is required" error; modal stays open</v>
+      </c>
+      <c r="R38" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S38" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B39" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C39" t="str">
+        <v>TC-AU-018</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Partner User without customer shows validation error</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F39" t="str">
+        <v>API</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H39" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I39" t="str">
+        <v>BUG-ADDNEWUSER-037</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Partner User without customer shows validation error</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L39" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M39" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select Partner User role
+2. Leave Customer empty
+3. Submit
+4. Check customer error</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>"Please select a customer" shown; modal stays open</v>
+      </c>
+      <c r="R39" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S39" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B40" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C40" t="str">
+        <v>TC-AU-015</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Duplicate username — silent failure BUG-AU-001</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F40" t="str">
+        <v>API</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H40" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I40" t="str">
+        <v>BUG-ADDNEWUSER-038</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Duplicate username — silent failure BUG-AU-001</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L40" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M40" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P40" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter existing username
+2. Submit
+3. Look for duplicate error message — currently none shown (BUG-AU-001)</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>Duplicate username rejected; error message "Username already taken" shown on form</v>
+      </c>
+      <c r="R40" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S40" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B41" t="str">
+        <v>AddNewUser</v>
+      </c>
+      <c r="C41" t="str">
+        <v>TC-AU-021</v>
+      </c>
+      <c r="D41" t="str">
+        <v>XSS payload in First Name does not execute</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F41" t="str">
+        <v>API</v>
+      </c>
+      <c r="G41" t="str">
+        <v>High</v>
+      </c>
+      <c r="H41" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I41" t="str">
+        <v>BUG-ADDNEWUSER-039</v>
+      </c>
+      <c r="J41" t="str">
+        <v>XSS payload in First Name does not execute</v>
+      </c>
+      <c r="K41" t="str">
+        <v>High</v>
+      </c>
+      <c r="L41" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M41" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N41" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O41" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P41" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter XSS in First Name
+2. Submit
+3. Check if alert fires</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>XSS payload not executed; alertFired=false; no script injection</v>
+      </c>
+      <c r="R41" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S41" t="str">
+        <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-07-01 18:04]:  — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S42"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2918,9 +2918,68 @@
         <v>Test Execution Report\Feature Reports\AddNewUser.xlsx</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v>-summary</v>
+      </c>
+      <c r="D42" t="str">
+        <v>All 0 TCs passed —  module</v>
+      </c>
+      <c r="E42" t="str">
+        <v>All types</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Unit / API / Auto</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Critical–Low</v>
+      </c>
+      <c r="H42" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I42" t="str">
+        <v>—</v>
+      </c>
+      <c r="J42" t="str">
+        <v>No bugs — 0/0 TCs passed</v>
+      </c>
+      <c r="K42" t="str">
+        <v>—</v>
+      </c>
+      <c r="L42" t="str">
+        <v>—</v>
+      </c>
+      <c r="M42" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N42" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O42" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P42" t="str">
+        <v>0 TCs via Playwright (tests/.spec.js)</v>
+      </c>
+      <c r="Q42" t="str">
+        <v>All 0 TCs pass</v>
+      </c>
+      <c r="R42" t="str">
+        <v>0/0 PASS ✓  Pass Rate: 100%</v>
+      </c>
+      <c r="S42" t="str">
+        <v>Test Execution Report\Feature Reports\.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S42"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Regression [Nightly 2026-07-01 20:22]: all — reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_01-Jul-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S53"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2977,9 +2977,680 @@
         <v>Test Execution Report\Feature Reports\.xlsx</v>
       </c>
     </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B43" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C43" t="str">
+        <v>TC-AQ-001</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Page loads with heading and pending items</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H43" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I43" t="str">
+        <v>BUG-ACTIONQUEUE-040</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Page loads with heading and pending items</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L43" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M43" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N43" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O43" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P43" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-AQ-001
+3. Observe failure</v>
+      </c>
+      <c r="Q43" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R43" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('text=7 Pending Actions') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('text=7 Pending Actions')</v>
+      </c>
+      <c r="S43" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B44" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C44" t="str">
+        <v>TC-AQ-012</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Search filters grid to matching rows</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H44" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I44" t="str">
+        <v>BUG-ACTIONQUEUE-041</v>
+      </c>
+      <c r="J44" t="str">
+        <v>Search filters grid to matching rows</v>
+      </c>
+      <c r="K44" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L44" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M44" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N44" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O44" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P44" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-AQ-012
+3. Observe failure</v>
+      </c>
+      <c r="Q44" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R44" t="str">
+        <v>Error: expect(received).toBeGreaterThanOrEqual(expected) Expected: &gt;= 1 Received: 0</v>
+      </c>
+      <c r="S44" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B45" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C45" t="str">
+        <v>TC-AQ-021</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Single character remarks accepted</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F45" t="str">
+        <v>API</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H45" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I45" t="str">
+        <v>BUG-ACTIONQUEUE-042</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Single character remarks accepted</v>
+      </c>
+      <c r="K45" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L45" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M45" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N45" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O45" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P45" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-AQ-021
+3. Observe failure</v>
+      </c>
+      <c r="Q45" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R45" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S45" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B46" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C46" t="str">
+        <v>TC-AQ-013</v>
+      </c>
+      <c r="D46" t="str">
+        <v>BACK button navigates away from detail page</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H46" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I46" t="str">
+        <v>BUG-ACTIONQUEUE-043</v>
+      </c>
+      <c r="J46" t="str">
+        <v>BACK button navigates away from detail page</v>
+      </c>
+      <c r="K46" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L46" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M46" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N46" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O46" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P46" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-AQ-013
+3. Observe failure</v>
+      </c>
+      <c r="Q46" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R46" t="str">
+        <v>Error: expect(received).not.toMatch(expected) Expected pattern: not /ActionQueueDetails/ Received string: "http://customerportal.dev-ts.online/Ticket/ActionQueueDetails/1345"</v>
+      </c>
+      <c r="S46" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B47" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C47" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="D47" t="str">
+        <v>All 4 stat cards visible with values</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H47" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I47" t="str">
+        <v>BUG-ACTIONQUEUE-044</v>
+      </c>
+      <c r="J47" t="str">
+        <v>All 4 stat cards visible with values</v>
+      </c>
+      <c r="K47" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L47" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M47" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N47" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O47" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P47" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-002
+3. Observe failure</v>
+      </c>
+      <c r="Q47" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R47" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S47" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B48" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C48" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="D48" t="str">
+        <v>ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H48" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I48" t="str">
+        <v>BUG-ACTIONQUEUE-045</v>
+      </c>
+      <c r="J48" t="str">
+        <v>ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="K48" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L48" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M48" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N48" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O48" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P48" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-004
+3. Observe failure</v>
+      </c>
+      <c r="Q48" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R48" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S48" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B49" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C49" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F49" t="str">
+        <v>API</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H49" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I49" t="str">
+        <v>BUG-ACTIONQUEUE-046</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="K49" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L49" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M49" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N49" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O49" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P49" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-005
+3. Observe failure</v>
+      </c>
+      <c r="Q49" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R49" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S49" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B50" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C50" t="str">
+        <v>TC-DASH-006</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Date range filter applies correctly</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F50" t="str">
+        <v>API</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H50" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I50" t="str">
+        <v>BUG-ACTIONQUEUE-047</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Date range filter applies correctly</v>
+      </c>
+      <c r="K50" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L50" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M50" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N50" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O50" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P50" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-006
+3. Observe failure</v>
+      </c>
+      <c r="Q50" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R50" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-07-02" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+      </c>
+      <c r="S50" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B51" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C51" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Reset button clears date filter</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F51" t="str">
+        <v>API</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H51" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I51" t="str">
+        <v>BUG-ACTIONQUEUE-048</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Reset button clears date filter</v>
+      </c>
+      <c r="K51" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L51" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M51" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N51" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O51" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P51" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-007
+3. Observe failure</v>
+      </c>
+      <c r="Q51" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R51" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-07-02" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+      </c>
+      <c r="S51" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B52" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C52" t="str">
+        <v>TC-DASH-008</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Invalid date range To &lt; From handled gracefully</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F52" t="str">
+        <v>API</v>
+      </c>
+      <c r="G52" t="str">
+        <v>High</v>
+      </c>
+      <c r="H52" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I52" t="str">
+        <v>BUG-ACTIONQUEUE-049</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Invalid date range To &lt; From handled gracefully</v>
+      </c>
+      <c r="K52" t="str">
+        <v>High</v>
+      </c>
+      <c r="L52" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M52" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N52" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O52" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P52" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-008
+3. Observe failure</v>
+      </c>
+      <c r="Q52" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R52" t="str">
+        <v>TimeoutError: locator.click: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_apply') - locator resolved to &lt;button id="dr_apply" class="w-full text-[0.75rem] font-bold text-white bg-blue-600 hover:bg-blue-700 rounded py-1.5 transition-colors"&gt;Apply Range&lt;/button&gt; - attempting click ac</v>
+      </c>
+      <c r="S52" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53" t="str">
+        <v>01 Jul 2026</v>
+      </c>
+      <c r="B53" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C53" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="D53" t="str">
+        <v>All sidebar navigation links present</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F53" t="str">
+        <v>API</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H53" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I53" t="str">
+        <v>BUG-ACTIONQUEUE-050</v>
+      </c>
+      <c r="J53" t="str">
+        <v>All sidebar navigation links present</v>
+      </c>
+      <c r="K53" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L53" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M53" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N53" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O53" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P53" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to ActionQueue feature
+2. Execute: TC-DASH-011
+3. Observe failure</v>
+      </c>
+      <c r="Q53" t="str">
+        <v>All Playwright assertions should pass</v>
+      </c>
+      <c r="R53" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('a[href="/Ticket/Index"]').first() 14 × locator resolved to &lt;a data-id="4" tab</v>
+      </c>
+      <c r="S53" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>